<commit_message>
fix: use defined named range =Ders_Listesi for subject validation dropdown
</commit_message>
<xml_diff>
--- a/YKS_2027_Calisma_Programi.xlsx
+++ b/YKS_2027_Calisma_Programi.xlsx
@@ -59218,76 +59218,76 @@
   </conditionalFormatting>
   <dataValidations count="48">
     <dataValidation type="list" allowBlank="1" sqref="B10">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B12">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B15">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B17">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B19">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B21">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B24">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B26">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B28">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B30">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B33">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B35">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B37">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B39">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B42">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B44">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B46">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B48">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B51">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B53">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B55">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B57">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B6">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B8">
-      <formula1>"TYT Türkçe,TYT-AYT Tarih,TYT Coğrafya,AYT Coğrafya,TYT Matematik,TYT Biyoloji,TYT Fizik,TYT Kimya,AYT Edebiyat"</formula1>
+      <formula1>=Ders_Listesi</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="C10">
       <formula1>=INDIRECT(SUBSTITUTE(SUBSTITUTE(B10," ","_"),"-","_"))</formula1>

</xml_diff>